<commit_message>
fix(varredura): suporte a novos dias no backfill e recuperacao de vendas da loja 19891 em 18/09
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-14).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-14).xlsx
@@ -959,10 +959,10 @@
     <t>6.1</t>
   </si>
   <si>
-    <t>40.5%</t>
-  </si>
-  <si>
-    <t>20.2%</t>
+    <t>40.3%</t>
+  </si>
+  <si>
+    <t>20.1%</t>
   </si>
   <si>
     <t>1.9%</t>
@@ -974,7 +974,7 @@
     <t>4.7%</t>
   </si>
   <si>
-    <t>1.5%</t>
+    <t>1.4%</t>
   </si>
   <si>
     <t>0.2%</t>
@@ -983,16 +983,16 @@
     <t>8.0%</t>
   </si>
   <si>
-    <t>3.4%</t>
+    <t>3.3%</t>
   </si>
   <si>
     <t>4.4%</t>
   </si>
   <si>
-    <t>1092.0</t>
-  </si>
-  <si>
-    <t>889.0</t>
+    <t>1094.0</t>
+  </si>
+  <si>
+    <t>891.0</t>
   </si>
   <si>
     <t>85.0</t>
@@ -1010,7 +1010,7 @@
     <t>8.0</t>
   </si>
   <si>
-    <t>351.0</t>
+    <t>353.0</t>
   </si>
   <si>
     <t>148.0</t>
@@ -7649,7 +7649,9 @@
       <c r="N42" s="6">
         <v>34</v>
       </c>
-      <c r="O42" s="6"/>
+      <c r="O42" s="6">
+        <v>24</v>
+      </c>
       <c r="P42" s="7">
         <v>5.2371428571428575</v>
       </c>
@@ -7659,31 +7661,75 @@
       <c r="R42" s="8">
         <v>6.4022727272727273</v>
       </c>
-      <c r="S42" s="8"/>
+      <c r="S42" s="8">
+        <v>7</v>
+      </c>
       <c r="T42" s="9">
         <v>0.33333333333333331</v>
       </c>
-      <c r="U42" s="9"/>
-      <c r="V42" s="9"/>
-      <c r="W42" s="9"/>
-      <c r="X42" s="9"/>
-      <c r="Y42" s="9"/>
-      <c r="Z42" s="9"/>
-      <c r="AA42" s="9"/>
-      <c r="AB42" s="9"/>
-      <c r="AC42" s="9"/>
-      <c r="AD42" s="6"/>
-      <c r="AE42" s="6"/>
-      <c r="AF42" s="6"/>
-      <c r="AG42" s="6"/>
-      <c r="AH42" s="6"/>
-      <c r="AI42" s="6"/>
-      <c r="AJ42" s="6"/>
-      <c r="AK42" s="6"/>
-      <c r="AL42" s="6"/>
-      <c r="AM42" s="6"/>
-      <c r="AN42" s="9"/>
-      <c r="AO42" s="6"/>
+      <c r="U42" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="V42" s="9">
+        <v>0</v>
+      </c>
+      <c r="W42" s="9">
+        <v>0</v>
+      </c>
+      <c r="X42" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="AB42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD42" s="6">
+        <v>2</v>
+      </c>
+      <c r="AE42" s="6">
+        <v>2</v>
+      </c>
+      <c r="AF42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK42" s="6">
+        <v>2</v>
+      </c>
+      <c r="AL42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO42" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP42" s="4">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
data: atualizacao da varredura com backfill e vendas ate 24/09
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-14).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-14).xlsx
@@ -935,19 +935,19 @@
     <t>214</t>
   </si>
   <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>R$ 3.264,92</t>
+    <t>27</t>
+  </si>
+  <si>
+    <t>R$ 3.264,53</t>
   </si>
   <si>
     <t>37.2</t>
   </si>
   <si>
-    <t>24.3</t>
-  </si>
-  <si>
-    <t>4.84</t>
+    <t>24.2</t>
+  </si>
+  <si>
+    <t>4.83</t>
   </si>
   <si>
     <t>19.3</t>
@@ -956,10 +956,10 @@
     <t>7.9</t>
   </si>
   <si>
-    <t>6.1</t>
-  </si>
-  <si>
-    <t>40.3%</t>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>40.6%</t>
   </si>
   <si>
     <t>20.1%</t>
@@ -10057,7 +10057,7 @@
         <v>19618</v>
       </c>
       <c r="B58" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C58" s="4">
         <v>51</v>
@@ -10087,14 +10087,26 @@
         <v>58</v>
       </c>
       <c r="L58" s="4"/>
-      <c r="M58" s="5"/>
-      <c r="N58" s="6"/>
+      <c r="M58" s="5">
+        <v>3193.1900000000001</v>
+      </c>
+      <c r="N58" s="6">
+        <v>37</v>
+      </c>
       <c r="O58" s="6"/>
-      <c r="P58" s="7"/>
-      <c r="Q58" s="8"/>
-      <c r="R58" s="8"/>
+      <c r="P58" s="7">
+        <v>3.3421052631578947</v>
+      </c>
+      <c r="Q58" s="8">
+        <v>17.541667647058823</v>
+      </c>
+      <c r="R58" s="8">
+        <v>7.3916676470588234</v>
+      </c>
       <c r="S58" s="8"/>
-      <c r="T58" s="9"/>
+      <c r="T58" s="9">
+        <v>0.5</v>
+      </c>
       <c r="U58" s="9"/>
       <c r="V58" s="9"/>
       <c r="W58" s="9"/>
@@ -17906,7 +17918,9 @@
       <c r="N111" s="6">
         <v>3</v>
       </c>
-      <c r="O111" s="6"/>
+      <c r="O111" s="6">
+        <v>3</v>
+      </c>
       <c r="P111" s="7">
         <v>6.8777666666666661</v>
       </c>
@@ -17916,31 +17930,75 @@
       <c r="R111" s="8">
         <v>2.3166666666666669</v>
       </c>
-      <c r="S111" s="8"/>
+      <c r="S111" s="8">
+        <v>7</v>
+      </c>
       <c r="T111" s="9">
         <v>0.33333333333333331</v>
       </c>
-      <c r="U111" s="9"/>
-      <c r="V111" s="9"/>
-      <c r="W111" s="9"/>
-      <c r="X111" s="9"/>
-      <c r="Y111" s="9"/>
-      <c r="Z111" s="9"/>
-      <c r="AA111" s="9"/>
-      <c r="AB111" s="9"/>
-      <c r="AC111" s="9"/>
-      <c r="AD111" s="6"/>
-      <c r="AE111" s="6"/>
-      <c r="AF111" s="6"/>
-      <c r="AG111" s="6"/>
-      <c r="AH111" s="6"/>
-      <c r="AI111" s="6"/>
-      <c r="AJ111" s="6"/>
-      <c r="AK111" s="6"/>
-      <c r="AL111" s="6"/>
-      <c r="AM111" s="6"/>
-      <c r="AN111" s="9"/>
-      <c r="AO111" s="6"/>
+      <c r="U111" s="9">
+        <v>0</v>
+      </c>
+      <c r="V111" s="9">
+        <v>0</v>
+      </c>
+      <c r="W111" s="9">
+        <v>0</v>
+      </c>
+      <c r="X111" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y111" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z111" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA111" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB111" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC111" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM111" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN111" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO111" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP111" s="4">
         <v>58</v>
       </c>

</xml_diff>